<commit_message>
Mull-Trans: raspored za Viljevo, Magadenovac, Podravsku Moslavinu i Košku završava kad ih preuzme novi davatelj
Od datuma kad počinje objavljeni raspored Doroslova (Viljevo 7.7.,
Magadenovac 3.9., Podravska Moslavina 7.9.) odnosno Urbanizma Valpovo
(Koška 8.10.) Mull-Transovi datumi se ne upisuju, pa za isti dan nema dva
rasporeda; napomena zone navodi novog davatelja.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012grr9UJafq4ZimrFiB6wUv
</commit_message>
<xml_diff>
--- a/excel/mull-trans/Pregled_zona.xlsx
+++ b/excel/mull-trans/Pregled_zona.xlsx
@@ -2520,7 +2520,7 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>2026: 39</t>
+          <t>2026: 30</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr"/>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>2026: 54</t>
+          <t>2026: 35</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr"/>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>2026: 53</t>
+          <t>2026: 36</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr"/>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>2026: 53</t>
+          <t>2026: 27</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr"/>

</xml_diff>